<commit_message>
Updated DZA_grids model - 2025-09-22 23:46
</commit_message>
<xml_diff>
--- a/VerveStacks_DZA_grids/Sets-vervestacks.xlsx
+++ b/VerveStacks_DZA_grids/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_DZA_grids\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C7F2C3D7-DC51-4498-81E8-4F0E5A881563}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{482E439A-5A06-41F1-9448-E74C572FC8F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2315,7 +2315,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F022F03-9208-4B44-879D-4E1F5724AB4E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D77C16F-B2E2-47BE-93D1-18291BABEA2C}">
   <dimension ref="B9:E198"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>